<commit_message>
update After show report
</commit_message>
<xml_diff>
--- a/Phase3EFMVCAPI/MeterManagement.API/file.xlsx
+++ b/Phase3EFMVCAPI/MeterManagement.API/file.xlsx
@@ -27,12 +27,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>SerialNumber</t>
   </si>
   <si>
-    <t>MTR0031</t>
+    <t>MTR0090</t>
+  </si>
+  <si>
+    <t>MTR0092</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1001,9 @@
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="2"/>
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="2"/>

</xml_diff>